<commit_message>
Add FTMO 100k account support, separate database files, and implement The5ers proxy crawl with premium token popup
</commit_message>
<xml_diff>
--- a/data/FTMO_10k.xlsx
+++ b/data/FTMO_10k.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="238">
   <si>
     <t>Mã số giao dịch</t>
   </si>
@@ -59,18 +59,81 @@
     <t>Thời lượng giao dịch tính bằng giây</t>
   </si>
   <si>
+    <t>146160046</t>
+  </si>
+  <si>
+    <t>2026-06-30 17:07:14</t>
+  </si>
+  <si>
+    <t>sell</t>
+  </si>
+  <si>
+    <t>BTCUSD</t>
+  </si>
+  <si>
+    <t>2026-07-01 04:39:30</t>
+  </si>
+  <si>
+    <t>145615795</t>
+  </si>
+  <si>
+    <t>2026-06-29 13:00:00</t>
+  </si>
+  <si>
+    <t>buy</t>
+  </si>
+  <si>
+    <t>USDJPY</t>
+  </si>
+  <si>
+    <t>2026-06-30 18:40:35</t>
+  </si>
+  <si>
+    <t>143893593</t>
+  </si>
+  <si>
+    <t>2026-06-23 15:02:05</t>
+  </si>
+  <si>
+    <t>GBPUSD</t>
+  </si>
+  <si>
+    <t>2026-06-25 16:21:24</t>
+  </si>
+  <si>
+    <t>143893506</t>
+  </si>
+  <si>
+    <t>2026-06-23 15:01:51</t>
+  </si>
+  <si>
+    <t>2026-06-23 15:01:55</t>
+  </si>
+  <si>
+    <t>141152513</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:38:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 21:17:30</t>
+  </si>
+  <si>
+    <t>141152493</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:37:53</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:37:57</t>
+  </si>
+  <si>
     <t>137218824</t>
   </si>
   <si>
     <t>2026-06-01 05:03:21</t>
   </si>
   <si>
-    <t>sell</t>
-  </si>
-  <si>
-    <t>BTCUSD</t>
-  </si>
-  <si>
     <t>2026-06-01 16:55:19</t>
   </si>
   <si>
@@ -110,12 +173,6 @@
     <t>2026-05-07 13:48:51</t>
   </si>
   <si>
-    <t>buy</t>
-  </si>
-  <si>
-    <t>GBPUSD</t>
-  </si>
-  <si>
     <t>2026-05-07 14:14:11</t>
   </si>
   <si>
@@ -222,9 +279,6 @@
   </si>
   <si>
     <t>2026-04-22 16:46:16</t>
-  </si>
-  <si>
-    <t>USDJPY</t>
   </si>
   <si>
     <t>2026-04-22 17:45:26</t>
@@ -1017,7 +1071,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18.71" bestFit="true" customWidth="true" style="0"/>
@@ -1095,40 +1149,40 @@
         <v>17</v>
       </c>
       <c r="D2" s="2">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="E2" t="s">
         <v>18</v>
       </c>
       <c r="F2" s="2">
-        <v>73313.52</v>
+        <v>58999.99</v>
       </c>
       <c r="G2" s="2">
-        <v>73282.85</v>
+        <v>58908.17</v>
       </c>
       <c r="H2" s="2">
-        <v>71436.33</v>
+        <v>55666.06</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="J2" s="2">
-        <v>71433.2</v>
+        <v>58882.78</v>
       </c>
       <c r="K2" s="2">
-        <v>0</v>
+        <v>-2.94</v>
       </c>
       <c r="L2" s="2">
-        <v>-5.17</v>
+        <v>-2.3</v>
       </c>
       <c r="M2" s="2">
-        <v>206.84</v>
+        <v>7.03</v>
       </c>
       <c r="N2" s="2">
-        <v>1880.3</v>
+        <v>117.2</v>
       </c>
       <c r="O2" s="3">
-        <v>42718</v>
+        <v>41536</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -1139,184 +1193,178 @@
         <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2">
-        <v>0.02</v>
+        <v>0.44</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3" s="2">
-        <v>4510.65</v>
+        <v>161.889</v>
       </c>
       <c r="G3" s="2">
-        <v>4508.54</v>
+        <v>161.911</v>
       </c>
       <c r="H3" s="2">
-        <v>4405.12</v>
+        <v>162.645</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" s="2">
-        <v>4404.3</v>
+        <v>162.62</v>
       </c>
       <c r="K3" s="2">
-        <v>0.17</v>
+        <v>1.02</v>
       </c>
       <c r="L3" s="2">
-        <v>-0.12</v>
+        <v>-2.2</v>
       </c>
       <c r="M3" s="2">
-        <v>212.7</v>
+        <v>197.79</v>
       </c>
       <c r="N3" s="2">
-        <v>106.4</v>
+        <v>73.1</v>
       </c>
       <c r="O3" s="3">
-        <v>90935</v>
+        <v>106835</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="2">
-        <v>0.02</v>
+        <v>0.18</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F4" s="2">
-        <v>4512.49</v>
+        <v>1.32147</v>
       </c>
       <c r="G4" s="2">
-        <v>4561.77</v>
+        <v>1.31965</v>
       </c>
       <c r="H4" s="2">
-        <v>4377.57</v>
+        <v>1.30477</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J4" s="2">
-        <v>4520.29</v>
+        <v>1.31874</v>
       </c>
       <c r="K4" s="2">
-        <v>0</v>
+        <v>-4.06</v>
       </c>
       <c r="L4" s="2">
-        <v>-0.12</v>
+        <v>-0.9</v>
       </c>
       <c r="M4" s="2">
-        <v>-15.6</v>
+        <v>49.14</v>
       </c>
       <c r="N4" s="2">
-        <v>-7.8</v>
+        <v>27.3</v>
       </c>
       <c r="O4" s="3">
-        <v>16327</v>
+        <v>177559</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="2">
-        <v>0.02</v>
+        <v>0.18</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F5" s="2">
-        <v>4674.88</v>
-      </c>
-      <c r="G5" s="2">
-        <v>4672.82</v>
-      </c>
-      <c r="H5" s="2">
-        <v>4573.56</v>
+        <v>62494.71</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J5" s="2">
-        <v>4573.31</v>
+        <v>62499.43</v>
       </c>
       <c r="K5" s="2">
-        <v>-0.11</v>
+        <v>0</v>
       </c>
       <c r="L5" s="2">
-        <v>-0.13</v>
+        <v>-7.32</v>
       </c>
       <c r="M5" s="2">
-        <v>203.14</v>
+        <v>-0.85</v>
       </c>
       <c r="N5" s="2">
-        <v>101.6</v>
+        <v>-4.7</v>
       </c>
       <c r="O5" s="3">
-        <v>91993</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2">
-        <v>0.5</v>
+        <v>0.06</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="F6" s="2">
-        <v>1.36231</v>
+        <v>63704.62</v>
       </c>
       <c r="G6" s="2">
-        <v>1.36133</v>
+        <v>62188.79</v>
       </c>
       <c r="H6" s="2">
-        <v>1.36437</v>
+        <v>67271.63</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="2">
-        <v>1.36133</v>
+        <v>63750.19</v>
       </c>
       <c r="K6" s="2">
         <v>0</v>
       </c>
       <c r="L6" s="2">
-        <v>-2.5</v>
+        <v>-2.48</v>
       </c>
       <c r="M6" s="2">
-        <v>-49.0</v>
+        <v>2.73</v>
       </c>
       <c r="N6" s="2">
-        <v>0</v>
+        <v>45.6</v>
       </c>
       <c r="O6" s="3">
-        <v>1520</v>
+        <v>27570</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -1330,40 +1378,34 @@
         <v>17</v>
       </c>
       <c r="D7" s="2">
-        <v>0.5</v>
+        <v>0.06</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="F7" s="2">
-        <v>1.35954</v>
-      </c>
-      <c r="G7" s="2">
-        <v>1.36051</v>
-      </c>
-      <c r="H7" s="2">
-        <v>1.35747</v>
+        <v>63690.2</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J7" s="2">
-        <v>1.36064</v>
+        <v>63695.3</v>
       </c>
       <c r="K7" s="2">
         <v>0</v>
       </c>
       <c r="L7" s="2">
-        <v>-2.5</v>
+        <v>-2.48</v>
       </c>
       <c r="M7" s="2">
-        <v>-55.0</v>
+        <v>-0.31</v>
       </c>
       <c r="N7" s="2">
-        <v>0</v>
+        <v>-5.1</v>
       </c>
       <c r="O7" s="3">
-        <v>2411</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -1374,43 +1416,43 @@
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2">
-        <v>0.5</v>
+        <v>0.11</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="F8" s="2">
-        <v>1.36006</v>
+        <v>73313.52</v>
       </c>
       <c r="G8" s="2">
-        <v>1.35908</v>
+        <v>73282.85</v>
       </c>
       <c r="H8" s="2">
-        <v>1.36213</v>
+        <v>71436.33</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="J8" s="2">
-        <v>1.35908</v>
+        <v>71433.2</v>
       </c>
       <c r="K8" s="2">
         <v>0</v>
       </c>
       <c r="L8" s="2">
-        <v>-2.5</v>
+        <v>-5.17</v>
       </c>
       <c r="M8" s="2">
-        <v>-49.0</v>
+        <v>206.84</v>
       </c>
       <c r="N8" s="2">
-        <v>0</v>
+        <v>1880.3</v>
       </c>
       <c r="O8" s="3">
-        <v>9731</v>
+        <v>42718</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -1421,463 +1463,463 @@
         <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D9" s="2">
-        <v>0.38</v>
+        <v>0.02</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F9" s="2">
-        <v>1.35502</v>
+        <v>4510.65</v>
       </c>
       <c r="G9" s="2">
-        <v>1.35373</v>
+        <v>4508.54</v>
       </c>
       <c r="H9" s="2">
-        <v>1.35805</v>
+        <v>4405.12</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J9" s="2">
-        <v>1.35771</v>
+        <v>4404.3</v>
       </c>
       <c r="K9" s="2">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="L9" s="2">
-        <v>-1.9</v>
+        <v>-0.12</v>
       </c>
       <c r="M9" s="2">
-        <v>102.22</v>
+        <v>212.7</v>
       </c>
       <c r="N9" s="2">
-        <v>0</v>
+        <v>106.4</v>
       </c>
       <c r="O9" s="3">
-        <v>9621</v>
+        <v>90935</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="2">
-        <v>0.49</v>
+        <v>0.02</v>
       </c>
       <c r="E10" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F10" s="2">
-        <v>1.35339</v>
+        <v>4512.49</v>
       </c>
       <c r="G10" s="2">
-        <v>1.35469</v>
+        <v>4561.77</v>
+      </c>
+      <c r="H10" s="2">
+        <v>4377.57</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J10" s="2">
-        <v>1.35472</v>
+        <v>4520.29</v>
       </c>
       <c r="K10" s="2">
         <v>0</v>
       </c>
       <c r="L10" s="2">
-        <v>-2.46</v>
+        <v>-0.12</v>
       </c>
       <c r="M10" s="2">
-        <v>-65.17</v>
+        <v>-15.6</v>
       </c>
       <c r="N10" s="2">
-        <v>0</v>
+        <v>-7.8</v>
       </c>
       <c r="O10" s="3">
-        <v>899</v>
+        <v>16327</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="2">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F11" s="2">
-        <v>1.3522</v>
+        <v>4674.88</v>
       </c>
       <c r="G11" s="2">
-        <v>1.35318</v>
+        <v>4672.82</v>
       </c>
       <c r="H11" s="2">
-        <v>1.35012</v>
+        <v>4573.56</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J11" s="2">
-        <v>1.35324</v>
+        <v>4573.31</v>
       </c>
       <c r="K11" s="2">
-        <v>0</v>
+        <v>-0.11</v>
       </c>
       <c r="L11" s="2">
-        <v>-2.5</v>
+        <v>-0.13</v>
       </c>
       <c r="M11" s="2">
-        <v>-52.0</v>
+        <v>203.14</v>
       </c>
       <c r="N11" s="2">
-        <v>0</v>
+        <v>101.6</v>
       </c>
       <c r="O11" s="3">
-        <v>9108</v>
+        <v>91993</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D12" s="2">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F12" s="2">
-        <v>1.36108</v>
+        <v>1.36231</v>
       </c>
       <c r="G12" s="2">
-        <v>1.36115</v>
+        <v>1.36133</v>
       </c>
       <c r="H12" s="2">
-        <v>1.36319</v>
+        <v>1.36437</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J12" s="2">
-        <v>1.36115</v>
+        <v>1.36133</v>
       </c>
       <c r="K12" s="2">
         <v>0</v>
       </c>
       <c r="L12" s="2">
-        <v>-2.46</v>
+        <v>-2.5</v>
       </c>
       <c r="M12" s="2">
-        <v>3.43</v>
+        <v>-49.0</v>
       </c>
       <c r="N12" s="2">
         <v>0</v>
       </c>
       <c r="O12" s="3">
-        <v>2633</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D13" s="2">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F13" s="2">
-        <v>1.36061</v>
+        <v>1.35954</v>
       </c>
       <c r="G13" s="2">
+        <v>1.36051</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1.35747</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J13" s="2">
         <v>1.36064</v>
       </c>
-      <c r="H13" s="2">
-        <v>1.362</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="J13" s="2">
-        <v>1.36062</v>
-      </c>
       <c r="K13" s="2">
         <v>0</v>
       </c>
       <c r="L13" s="2">
-        <v>-4</v>
+        <v>-2.5</v>
       </c>
       <c r="M13" s="2">
-        <v>0.8</v>
+        <v>-55.0</v>
       </c>
       <c r="N13" s="2">
         <v>0</v>
       </c>
       <c r="O13" s="3">
-        <v>5896</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D14" s="2">
-        <v>0.56</v>
+        <v>0.5</v>
       </c>
       <c r="E14" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F14" s="2">
-        <v>1.35141</v>
+        <v>1.36006</v>
       </c>
       <c r="G14" s="2">
-        <v>1.35238</v>
+        <v>1.35908</v>
       </c>
       <c r="H14" s="2">
-        <v>1.34955</v>
+        <v>1.36213</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J14" s="2">
-        <v>1.34954</v>
+        <v>1.35908</v>
       </c>
       <c r="K14" s="2">
         <v>0</v>
       </c>
       <c r="L14" s="2">
-        <v>-2.8</v>
+        <v>-2.5</v>
       </c>
       <c r="M14" s="2">
-        <v>104.72</v>
+        <v>-49.0</v>
       </c>
       <c r="N14" s="2">
         <v>0</v>
       </c>
       <c r="O14" s="3">
-        <v>12842</v>
+        <v>9731</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D15" s="2">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="E15" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F15" s="2">
-        <v>1.35009</v>
+        <v>1.35502</v>
       </c>
       <c r="G15" s="2">
-        <v>1.35013</v>
+        <v>1.35373</v>
       </c>
       <c r="H15" s="2">
-        <v>1.35246</v>
+        <v>1.35805</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J15" s="2">
-        <v>1.35247</v>
+        <v>1.35771</v>
       </c>
       <c r="K15" s="2">
         <v>0</v>
       </c>
       <c r="L15" s="2">
-        <v>-2.16</v>
+        <v>-1.9</v>
       </c>
       <c r="M15" s="2">
-        <v>102.34</v>
+        <v>102.22</v>
       </c>
       <c r="N15" s="2">
         <v>0</v>
       </c>
       <c r="O15" s="3">
-        <v>11311</v>
+        <v>9621</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="2">
-        <v>0.32</v>
+        <v>0.49</v>
       </c>
       <c r="E16" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F16" s="2">
-        <v>1.34768</v>
+        <v>1.35339</v>
       </c>
       <c r="G16" s="2">
-        <v>1.35075</v>
-      </c>
-      <c r="H16" s="2">
-        <v>1.34111</v>
+        <v>1.35469</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J16" s="2">
-        <v>1.34996</v>
+        <v>1.35472</v>
       </c>
       <c r="K16" s="2">
-        <v>-2.12</v>
+        <v>0</v>
       </c>
       <c r="L16" s="2">
-        <v>-1.6</v>
+        <v>-2.46</v>
       </c>
       <c r="M16" s="2">
-        <v>-72.96</v>
+        <v>-65.17</v>
       </c>
       <c r="N16" s="2">
         <v>0</v>
       </c>
       <c r="O16" s="3">
-        <v>68328</v>
+        <v>899</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="2">
-        <v>0.31</v>
+        <v>0.5</v>
       </c>
       <c r="E17" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F17" s="2">
-        <v>1.34859</v>
+        <v>1.3522</v>
       </c>
       <c r="G17" s="2">
-        <v>1.35158</v>
+        <v>1.35318</v>
       </c>
       <c r="H17" s="2">
-        <v>1.3416</v>
+        <v>1.35012</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J17" s="2">
-        <v>1.35158</v>
+        <v>1.35324</v>
       </c>
       <c r="K17" s="2">
         <v>0</v>
       </c>
       <c r="L17" s="2">
-        <v>-1.56</v>
+        <v>-2.5</v>
       </c>
       <c r="M17" s="2">
-        <v>-92.69</v>
+        <v>-52.0</v>
       </c>
       <c r="N17" s="2">
         <v>0</v>
       </c>
       <c r="O17" s="3">
-        <v>13714</v>
+        <v>9108</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D18" s="2">
-        <v>0.7</v>
+        <v>0.49</v>
       </c>
       <c r="E18" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="F18" s="2">
-        <v>159.146</v>
+        <v>1.36108</v>
       </c>
       <c r="G18" s="2">
-        <v>159.366</v>
+        <v>1.36115</v>
       </c>
       <c r="H18" s="2">
-        <v>158.603</v>
+        <v>1.36319</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>71</v>
       </c>
       <c r="J18" s="2">
-        <v>159.273</v>
+        <v>1.36115</v>
       </c>
       <c r="K18" s="2">
         <v>0</v>
       </c>
       <c r="L18" s="2">
-        <v>-3.5</v>
+        <v>-2.46</v>
       </c>
       <c r="M18" s="2">
-        <v>-55.82</v>
+        <v>3.43</v>
       </c>
       <c r="N18" s="2">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="O18" s="3">
-        <v>3550</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1888,43 +1930,43 @@
         <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D19" s="2">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E19" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="F19" s="2">
-        <v>159.347</v>
+        <v>1.36061</v>
       </c>
       <c r="G19" s="2">
-        <v>159.125</v>
+        <v>1.36064</v>
       </c>
       <c r="H19" s="2">
-        <v>159.81</v>
+        <v>1.362</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>74</v>
       </c>
       <c r="J19" s="2">
-        <v>159.112</v>
+        <v>1.36062</v>
       </c>
       <c r="K19" s="2">
         <v>0</v>
       </c>
       <c r="L19" s="2">
-        <v>-3.5</v>
+        <v>-4</v>
       </c>
       <c r="M19" s="2">
-        <v>-103.39</v>
+        <v>0.8</v>
       </c>
       <c r="N19" s="2">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="O19" s="3">
-        <v>2354</v>
+        <v>5896</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1935,43 +1977,43 @@
         <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D20" s="2">
-        <v>0.27</v>
+        <v>0.56</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F20" s="2">
-        <v>1.35178</v>
+        <v>1.35141</v>
       </c>
       <c r="G20" s="2">
-        <v>1.34825</v>
+        <v>1.35238</v>
       </c>
       <c r="H20" s="2">
-        <v>1.35962</v>
+        <v>1.34955</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>77</v>
       </c>
       <c r="J20" s="2">
-        <v>1.34928</v>
+        <v>1.34954</v>
       </c>
       <c r="K20" s="2">
         <v>0</v>
       </c>
       <c r="L20" s="2">
-        <v>-1.36</v>
+        <v>-2.8</v>
       </c>
       <c r="M20" s="2">
-        <v>-67.5</v>
+        <v>104.72</v>
       </c>
       <c r="N20" s="2">
         <v>0</v>
       </c>
       <c r="O20" s="3">
-        <v>24249</v>
+        <v>12842</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -1982,43 +2024,43 @@
         <v>79</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D21" s="2">
-        <v>0.49</v>
+        <v>0.43</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="F21" s="2">
-        <v>158.859</v>
+        <v>1.35009</v>
       </c>
       <c r="G21" s="2">
-        <v>159.006</v>
+        <v>1.35013</v>
       </c>
       <c r="H21" s="2">
-        <v>159.517</v>
+        <v>1.35246</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J21" s="2">
-        <v>159.469</v>
+        <v>1.35247</v>
       </c>
       <c r="K21" s="2">
         <v>0</v>
       </c>
       <c r="L21" s="2">
-        <v>-2.46</v>
+        <v>-2.16</v>
       </c>
       <c r="M21" s="2">
-        <v>187.43</v>
+        <v>102.34</v>
       </c>
       <c r="N21" s="2">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="O21" s="3">
-        <v>60286</v>
+        <v>11311</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -2032,40 +2074,40 @@
         <v>17</v>
       </c>
       <c r="D22" s="2">
-        <v>0.01</v>
+        <v>0.32</v>
       </c>
       <c r="E22" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F22" s="2">
-        <v>4789.19</v>
+        <v>1.34768</v>
       </c>
       <c r="G22" s="2">
-        <v>4816.02</v>
+        <v>1.35075</v>
       </c>
       <c r="H22" s="2">
-        <v>4701.04</v>
+        <v>1.34111</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>83</v>
       </c>
       <c r="J22" s="2">
-        <v>4816.75</v>
+        <v>1.34996</v>
       </c>
       <c r="K22" s="2">
-        <v>0</v>
+        <v>-2.12</v>
       </c>
       <c r="L22" s="2">
-        <v>-0.06</v>
+        <v>-1.6</v>
       </c>
       <c r="M22" s="2">
-        <v>-27.56</v>
+        <v>-72.96</v>
       </c>
       <c r="N22" s="2">
-        <v>-27.6</v>
+        <v>0</v>
       </c>
       <c r="O22" s="3">
-        <v>37701</v>
+        <v>68328</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -2079,40 +2121,40 @@
         <v>17</v>
       </c>
       <c r="D23" s="2">
-        <v>0.02</v>
+        <v>0.31</v>
       </c>
       <c r="E23" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F23" s="2">
-        <v>4781.83</v>
+        <v>1.34859</v>
       </c>
       <c r="G23" s="2">
-        <v>4815.28</v>
+        <v>1.35158</v>
       </c>
       <c r="H23" s="2">
-        <v>4700.55</v>
+        <v>1.3416</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>86</v>
       </c>
       <c r="J23" s="2">
-        <v>4815.31</v>
+        <v>1.35158</v>
       </c>
       <c r="K23" s="2">
         <v>0</v>
       </c>
       <c r="L23" s="2">
-        <v>-0.14</v>
+        <v>-1.56</v>
       </c>
       <c r="M23" s="2">
-        <v>-66.96</v>
+        <v>-92.69</v>
       </c>
       <c r="N23" s="2">
-        <v>-33.5</v>
+        <v>0</v>
       </c>
       <c r="O23" s="3">
-        <v>38028</v>
+        <v>13714</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -2123,90 +2165,90 @@
         <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D24" s="2">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
       <c r="E24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="2">
+        <v>159.146</v>
+      </c>
+      <c r="G24" s="2">
+        <v>159.366</v>
+      </c>
+      <c r="H24" s="2">
+        <v>158.603</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F24" s="2">
-        <v>1.17904</v>
-      </c>
-      <c r="G24" s="2">
-        <v>1.1791</v>
-      </c>
-      <c r="H24" s="2">
-        <v>1.18335</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="J24" s="2">
-        <v>1.17942</v>
+        <v>159.273</v>
       </c>
       <c r="K24" s="2">
-        <v>-16.58</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2">
-        <v>-2.6</v>
+        <v>-3.5</v>
       </c>
       <c r="M24" s="2">
-        <v>19.76</v>
+        <v>-55.82</v>
       </c>
       <c r="N24" s="2">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="O24" s="3">
-        <v>63253</v>
+        <v>3550</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="2">
+        <v>159.347</v>
+      </c>
+      <c r="G25" s="2">
+        <v>159.125</v>
+      </c>
+      <c r="H25" s="2">
+        <v>159.81</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D25" s="2">
-        <v>0.55</v>
-      </c>
-      <c r="E25" t="s">
-        <v>70</v>
-      </c>
-      <c r="F25" s="2">
-        <v>158.79</v>
-      </c>
-      <c r="G25" s="2">
-        <v>159.066</v>
-      </c>
-      <c r="H25" s="2">
-        <v>158.204</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="J25" s="2">
-        <v>158.954</v>
+        <v>159.112</v>
       </c>
       <c r="K25" s="2">
         <v>0</v>
       </c>
       <c r="L25" s="2">
-        <v>-2.76</v>
+        <v>-3.5</v>
       </c>
       <c r="M25" s="2">
-        <v>-56.75</v>
+        <v>-103.39</v>
       </c>
       <c r="N25" s="2">
         <v>-0.2</v>
       </c>
       <c r="O25" s="3">
-        <v>21215</v>
+        <v>2354</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -2217,43 +2259,43 @@
         <v>94</v>
       </c>
       <c r="C26" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D26" s="2">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="E26" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F26" s="2">
-        <v>1.34201</v>
+        <v>1.35178</v>
       </c>
       <c r="G26" s="2">
-        <v>1.33874</v>
+        <v>1.34825</v>
       </c>
       <c r="H26" s="2">
-        <v>1.34828</v>
+        <v>1.35962</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>95</v>
       </c>
       <c r="J26" s="2">
-        <v>1.34233</v>
+        <v>1.34928</v>
       </c>
       <c r="K26" s="2">
-        <v>-1.68</v>
+        <v>0</v>
       </c>
       <c r="L26" s="2">
-        <v>-1.5</v>
+        <v>-1.36</v>
       </c>
       <c r="M26" s="2">
-        <v>9.6</v>
+        <v>-67.5</v>
       </c>
       <c r="N26" s="2">
         <v>0</v>
       </c>
       <c r="O26" s="3">
-        <v>49180</v>
+        <v>24249</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -2264,43 +2306,43 @@
         <v>97</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D27" s="2">
-        <v>0.02</v>
+        <v>0.49</v>
       </c>
       <c r="E27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F27" s="2">
-        <v>4743.05</v>
+        <v>158.859</v>
       </c>
       <c r="G27" s="2">
-        <v>4701.85</v>
+        <v>159.006</v>
       </c>
       <c r="H27" s="2">
-        <v>4854.69</v>
+        <v>159.517</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>98</v>
       </c>
       <c r="J27" s="2">
-        <v>4743.81</v>
+        <v>159.469</v>
       </c>
       <c r="K27" s="2">
-        <v>-1.81</v>
+        <v>0</v>
       </c>
       <c r="L27" s="2">
-        <v>-0.14</v>
+        <v>-2.46</v>
       </c>
       <c r="M27" s="2">
-        <v>1.52</v>
+        <v>187.43</v>
       </c>
       <c r="N27" s="2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O27" s="3">
-        <v>48672</v>
+        <v>60286</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -2311,43 +2353,43 @@
         <v>100</v>
       </c>
       <c r="C28" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D28" s="2">
-        <v>0.43</v>
+        <v>0.01</v>
       </c>
       <c r="E28" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F28" s="2">
-        <v>159.744</v>
+        <v>4789.19</v>
       </c>
       <c r="G28" s="2">
-        <v>159.761</v>
+        <v>4816.02</v>
       </c>
       <c r="H28" s="2">
-        <v>160.497</v>
+        <v>4701.04</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>101</v>
       </c>
       <c r="J28" s="2">
-        <v>159.754</v>
+        <v>4816.75</v>
       </c>
       <c r="K28" s="2">
         <v>0</v>
       </c>
       <c r="L28" s="2">
-        <v>-2.16</v>
+        <v>-0.06</v>
       </c>
       <c r="M28" s="2">
-        <v>2.69</v>
+        <v>-27.56</v>
       </c>
       <c r="N28" s="2">
-        <v>0</v>
+        <v>-27.6</v>
       </c>
       <c r="O28" s="3">
-        <v>45133</v>
+        <v>37701</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -2358,43 +2400,43 @@
         <v>103</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D29" s="2">
-        <v>0.28</v>
+        <v>0.02</v>
       </c>
       <c r="E29" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F29" s="2">
-        <v>1.32545</v>
+        <v>4781.83</v>
       </c>
       <c r="G29" s="2">
-        <v>1.32196</v>
+        <v>4815.28</v>
       </c>
       <c r="H29" s="2">
-        <v>1.34089</v>
+        <v>4700.55</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>104</v>
       </c>
       <c r="J29" s="2">
-        <v>1.33228</v>
+        <v>4815.31</v>
       </c>
       <c r="K29" s="2">
         <v>0</v>
       </c>
       <c r="L29" s="2">
-        <v>-1.4</v>
+        <v>-0.14</v>
       </c>
       <c r="M29" s="2">
-        <v>191.24</v>
+        <v>-66.96</v>
       </c>
       <c r="N29" s="2">
-        <v>0</v>
+        <v>-33.5</v>
       </c>
       <c r="O29" s="3">
-        <v>23627</v>
+        <v>38028</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -2405,90 +2447,90 @@
         <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D30" s="2">
-        <v>0.26</v>
+        <v>0.52</v>
       </c>
       <c r="E30" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="F30" s="2">
-        <v>159.21</v>
+        <v>1.17904</v>
       </c>
       <c r="G30" s="2">
-        <v>159.258</v>
+        <v>1.1791</v>
       </c>
       <c r="H30" s="2">
-        <v>159.951</v>
+        <v>1.18335</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J30" s="2">
-        <v>159.504</v>
+        <v>1.17942</v>
       </c>
       <c r="K30" s="2">
-        <v>2.14</v>
+        <v>-16.58</v>
       </c>
       <c r="L30" s="2">
-        <v>-1.3</v>
+        <v>-2.6</v>
       </c>
       <c r="M30" s="2">
-        <v>47.92</v>
+        <v>19.76</v>
       </c>
       <c r="N30" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="O30" s="3">
-        <v>119435</v>
+        <v>63253</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="2">
-        <v>0.49</v>
+        <v>0.55</v>
       </c>
       <c r="E31" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="F31" s="2">
-        <v>158.672</v>
+        <v>158.79</v>
       </c>
       <c r="G31" s="2">
-        <v>158.992</v>
+        <v>159.066</v>
       </c>
       <c r="H31" s="2">
-        <v>158.008</v>
+        <v>158.204</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J31" s="2">
-        <v>158.994</v>
+        <v>158.954</v>
       </c>
       <c r="K31" s="2">
         <v>0</v>
       </c>
       <c r="L31" s="2">
-        <v>-2.46</v>
+        <v>-2.76</v>
       </c>
       <c r="M31" s="2">
-        <v>-99.24</v>
+        <v>-56.75</v>
       </c>
       <c r="N31" s="2">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="O31" s="3">
-        <v>24549</v>
+        <v>21215</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -2499,40 +2541,43 @@
         <v>112</v>
       </c>
       <c r="C32" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D32" s="2">
-        <v>0.01</v>
+        <v>0.3</v>
       </c>
       <c r="E32" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F32" s="2">
-        <v>4426.13</v>
+        <v>1.34201</v>
       </c>
       <c r="G32" s="2">
-        <v>4351.51</v>
+        <v>1.33874</v>
+      </c>
+      <c r="H32" s="2">
+        <v>1.34828</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>113</v>
       </c>
       <c r="J32" s="2">
-        <v>4394.15</v>
+        <v>1.34233</v>
       </c>
       <c r="K32" s="2">
-        <v>0</v>
+        <v>-1.68</v>
       </c>
       <c r="L32" s="2">
-        <v>-0.06</v>
+        <v>-1.5</v>
       </c>
       <c r="M32" s="2">
-        <v>-31.98</v>
+        <v>9.6</v>
       </c>
       <c r="N32" s="2">
-        <v>-32</v>
+        <v>0</v>
       </c>
       <c r="O32" s="3">
-        <v>1391</v>
+        <v>49180</v>
       </c>
     </row>
     <row r="33" spans="1:15">
@@ -2543,43 +2588,43 @@
         <v>115</v>
       </c>
       <c r="C33" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D33" s="2">
-        <v>0.49</v>
+        <v>0.02</v>
       </c>
       <c r="E33" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F33" s="2">
-        <v>158.619</v>
+        <v>4743.05</v>
       </c>
       <c r="G33" s="2">
-        <v>158.926</v>
+        <v>4701.85</v>
       </c>
       <c r="H33" s="2">
-        <v>157.969</v>
+        <v>4854.69</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>116</v>
       </c>
       <c r="J33" s="2">
-        <v>158.806</v>
+        <v>4743.81</v>
       </c>
       <c r="K33" s="2">
-        <v>0</v>
+        <v>-1.81</v>
       </c>
       <c r="L33" s="2">
-        <v>-2.46</v>
+        <v>-0.14</v>
       </c>
       <c r="M33" s="2">
-        <v>-57.7</v>
+        <v>1.52</v>
       </c>
       <c r="N33" s="2">
-        <v>-0.2</v>
+        <v>0.8</v>
       </c>
       <c r="O33" s="3">
-        <v>3373</v>
+        <v>48672</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -2590,43 +2635,43 @@
         <v>118</v>
       </c>
       <c r="C34" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D34" s="2">
-        <v>0.49</v>
+        <v>0.43</v>
       </c>
       <c r="E34" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="F34" s="2">
-        <v>158.821</v>
+        <v>159.744</v>
       </c>
       <c r="G34" s="2">
-        <v>158.501</v>
+        <v>159.761</v>
       </c>
       <c r="H34" s="2">
-        <v>159.685</v>
+        <v>160.497</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>119</v>
       </c>
       <c r="J34" s="2">
-        <v>158.67</v>
+        <v>159.754</v>
       </c>
       <c r="K34" s="2">
         <v>0</v>
       </c>
       <c r="L34" s="2">
-        <v>-2.46</v>
+        <v>-2.16</v>
       </c>
       <c r="M34" s="2">
-        <v>-46.63</v>
+        <v>2.69</v>
       </c>
       <c r="N34" s="2">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="O34" s="3">
-        <v>4963</v>
+        <v>45133</v>
       </c>
     </row>
     <row r="35" spans="1:15">
@@ -2637,43 +2682,43 @@
         <v>121</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D35" s="2">
-        <v>0.01</v>
+        <v>0.28</v>
       </c>
       <c r="E35" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F35" s="2">
-        <v>4411.34</v>
+        <v>1.32545</v>
       </c>
       <c r="G35" s="2">
-        <v>4323.31</v>
+        <v>1.32196</v>
       </c>
       <c r="H35" s="2">
-        <v>4598.88</v>
+        <v>1.34089</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>122</v>
       </c>
       <c r="J35" s="2">
-        <v>4363.4</v>
+        <v>1.33228</v>
       </c>
       <c r="K35" s="2">
         <v>0</v>
       </c>
       <c r="L35" s="2">
-        <v>-0.06</v>
+        <v>-1.4</v>
       </c>
       <c r="M35" s="2">
-        <v>-47.94</v>
+        <v>191.24</v>
       </c>
       <c r="N35" s="2">
-        <v>-47.9</v>
+        <v>0</v>
       </c>
       <c r="O35" s="3">
-        <v>20356</v>
+        <v>23627</v>
       </c>
     </row>
     <row r="36" spans="1:15">
@@ -2684,43 +2729,43 @@
         <v>124</v>
       </c>
       <c r="C36" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D36" s="2">
-        <v>0.02</v>
+        <v>0.26</v>
       </c>
       <c r="E36" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F36" s="2">
-        <v>68514.6</v>
+        <v>159.21</v>
       </c>
       <c r="G36" s="2">
-        <v>73181.88</v>
+        <v>159.258</v>
       </c>
       <c r="H36" s="2">
-        <v>58231.26</v>
+        <v>159.951</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>125</v>
       </c>
       <c r="J36" s="2">
-        <v>71388.41</v>
+        <v>159.504</v>
       </c>
       <c r="K36" s="2">
-        <v>0</v>
+        <v>2.14</v>
       </c>
       <c r="L36" s="2">
-        <v>-0.91</v>
+        <v>-1.3</v>
       </c>
       <c r="M36" s="2">
-        <v>-57.48</v>
+        <v>47.92</v>
       </c>
       <c r="N36" s="2">
-        <v>-2873.8</v>
+        <v>0.3</v>
       </c>
       <c r="O36" s="3">
-        <v>19598</v>
+        <v>119435</v>
       </c>
     </row>
     <row r="37" spans="1:15">
@@ -2734,40 +2779,40 @@
         <v>17</v>
       </c>
       <c r="D37" s="2">
-        <v>0.32</v>
+        <v>0.49</v>
       </c>
       <c r="E37" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F37" s="2">
-        <v>1.32937</v>
+        <v>158.672</v>
       </c>
       <c r="G37" s="2">
-        <v>1.33244</v>
+        <v>158.992</v>
       </c>
       <c r="H37" s="2">
-        <v>1.32309</v>
+        <v>158.008</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>128</v>
       </c>
       <c r="J37" s="2">
-        <v>1.33244</v>
+        <v>158.994</v>
       </c>
       <c r="K37" s="2">
         <v>0</v>
       </c>
       <c r="L37" s="2">
-        <v>-1.6</v>
+        <v>-2.46</v>
       </c>
       <c r="M37" s="2">
-        <v>-98.24</v>
+        <v>-99.24</v>
       </c>
       <c r="N37" s="2">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="O37" s="3">
-        <v>4152</v>
+        <v>24549</v>
       </c>
     </row>
     <row r="38" spans="1:15">
@@ -2778,40 +2823,40 @@
         <v>130</v>
       </c>
       <c r="C38" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D38" s="2">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E38" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F38" s="2">
-        <v>4991.57</v>
+        <v>4426.13</v>
       </c>
       <c r="G38" s="2">
-        <v>5023.14</v>
+        <v>4351.51</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>131</v>
       </c>
       <c r="J38" s="2">
-        <v>4991.25</v>
+        <v>4394.15</v>
       </c>
       <c r="K38" s="2">
         <v>0</v>
       </c>
       <c r="L38" s="2">
-        <v>-0.2</v>
+        <v>-0.06</v>
       </c>
       <c r="M38" s="2">
-        <v>0.96</v>
+        <v>-31.98</v>
       </c>
       <c r="N38" s="2">
-        <v>0.3</v>
+        <v>-32</v>
       </c>
       <c r="O38" s="3">
-        <v>8972</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="39" spans="1:15">
@@ -2825,40 +2870,40 @@
         <v>17</v>
       </c>
       <c r="D39" s="2">
-        <v>0.02</v>
+        <v>0.49</v>
       </c>
       <c r="E39" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F39" s="2">
-        <v>4997.44</v>
+        <v>158.619</v>
       </c>
       <c r="G39" s="2">
-        <v>5021.56</v>
+        <v>158.926</v>
       </c>
       <c r="H39" s="2">
-        <v>4907.23</v>
+        <v>157.969</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>134</v>
       </c>
       <c r="J39" s="2">
-        <v>5004.36</v>
+        <v>158.806</v>
       </c>
       <c r="K39" s="2">
         <v>0</v>
       </c>
       <c r="L39" s="2">
-        <v>-0.14</v>
+        <v>-2.46</v>
       </c>
       <c r="M39" s="2">
-        <v>-13.84</v>
+        <v>-57.7</v>
       </c>
       <c r="N39" s="2">
-        <v>-6.9</v>
+        <v>-0.2</v>
       </c>
       <c r="O39" s="3">
-        <v>5470</v>
+        <v>3373</v>
       </c>
     </row>
     <row r="40" spans="1:15">
@@ -2869,43 +2914,43 @@
         <v>136</v>
       </c>
       <c r="C40" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D40" s="2">
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="E40" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="F40" s="2">
-        <v>159.217</v>
+        <v>158.821</v>
       </c>
       <c r="G40" s="2">
-        <v>159.205</v>
+        <v>158.501</v>
       </c>
       <c r="H40" s="2">
-        <v>158.671</v>
+        <v>159.685</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>137</v>
       </c>
       <c r="J40" s="2">
-        <v>158.748</v>
+        <v>158.67</v>
       </c>
       <c r="K40" s="2">
         <v>0</v>
       </c>
       <c r="L40" s="2">
-        <v>-3.26</v>
+        <v>-2.46</v>
       </c>
       <c r="M40" s="2">
-        <v>192.03</v>
+        <v>-46.63</v>
       </c>
       <c r="N40" s="2">
-        <v>0.5</v>
+        <v>-0.2</v>
       </c>
       <c r="O40" s="3">
-        <v>21651</v>
+        <v>4963</v>
       </c>
     </row>
     <row r="41" spans="1:15">
@@ -2916,43 +2961,43 @@
         <v>139</v>
       </c>
       <c r="C41" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D41" s="2">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E41" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F41" s="2">
-        <v>5013.0</v>
+        <v>4411.34</v>
       </c>
       <c r="G41" s="2">
-        <v>5036.01</v>
+        <v>4323.31</v>
       </c>
       <c r="H41" s="2">
-        <v>4938.12</v>
+        <v>4598.88</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>140</v>
       </c>
       <c r="J41" s="2">
-        <v>5021.27</v>
+        <v>4363.4</v>
       </c>
       <c r="K41" s="2">
         <v>0</v>
       </c>
       <c r="L41" s="2">
-        <v>-0.22</v>
+        <v>-0.06</v>
       </c>
       <c r="M41" s="2">
-        <v>-24.81</v>
+        <v>-47.94</v>
       </c>
       <c r="N41" s="2">
-        <v>-8.3</v>
+        <v>-47.9</v>
       </c>
       <c r="O41" s="3">
-        <v>12894</v>
+        <v>20356</v>
       </c>
     </row>
     <row r="42" spans="1:15">
@@ -2966,40 +3011,40 @@
         <v>17</v>
       </c>
       <c r="D42" s="2">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="E42" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F42" s="2">
-        <v>5009.64</v>
+        <v>68514.6</v>
       </c>
       <c r="G42" s="2">
-        <v>5039.17</v>
+        <v>73181.88</v>
       </c>
       <c r="H42" s="2">
-        <v>4945.32</v>
+        <v>58231.26</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>143</v>
       </c>
       <c r="J42" s="2">
-        <v>5023.34</v>
+        <v>71388.41</v>
       </c>
       <c r="K42" s="2">
         <v>0</v>
       </c>
       <c r="L42" s="2">
-        <v>-0.22</v>
+        <v>-0.91</v>
       </c>
       <c r="M42" s="2">
-        <v>-41.1</v>
+        <v>-57.48</v>
       </c>
       <c r="N42" s="2">
-        <v>-13.7</v>
+        <v>-2873.8</v>
       </c>
       <c r="O42" s="3">
-        <v>2006</v>
+        <v>19598</v>
       </c>
     </row>
     <row r="43" spans="1:15">
@@ -3010,43 +3055,43 @@
         <v>145</v>
       </c>
       <c r="C43" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D43" s="2">
-        <v>0.02</v>
+        <v>0.32</v>
       </c>
       <c r="E43" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F43" s="2">
-        <v>5032.46</v>
+        <v>1.32937</v>
       </c>
       <c r="G43" s="2">
-        <v>4996.97</v>
+        <v>1.33244</v>
       </c>
       <c r="H43" s="2">
-        <v>5120.3</v>
+        <v>1.32309</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>146</v>
       </c>
       <c r="J43" s="2">
-        <v>5007.9</v>
+        <v>1.33244</v>
       </c>
       <c r="K43" s="2">
         <v>0</v>
       </c>
       <c r="L43" s="2">
-        <v>-0.14</v>
+        <v>-1.6</v>
       </c>
       <c r="M43" s="2">
-        <v>-49.12</v>
+        <v>-98.24</v>
       </c>
       <c r="N43" s="2">
-        <v>-24.6</v>
+        <v>0</v>
       </c>
       <c r="O43" s="3">
-        <v>10248</v>
+        <v>4152</v>
       </c>
     </row>
     <row r="44" spans="1:15">
@@ -3060,40 +3105,37 @@
         <v>17</v>
       </c>
       <c r="D44" s="2">
-        <v>0.4</v>
+        <v>0.03</v>
       </c>
       <c r="E44" t="s">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="F44" s="2">
-        <v>1.14738</v>
+        <v>4991.57</v>
       </c>
       <c r="G44" s="2">
-        <v>1.1486</v>
-      </c>
-      <c r="H44" s="2">
-        <v>1.14474</v>
+        <v>5023.14</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>149</v>
       </c>
       <c r="J44" s="2">
-        <v>1.14861</v>
+        <v>4991.25</v>
       </c>
       <c r="K44" s="2">
         <v>0</v>
       </c>
       <c r="L44" s="2">
-        <v>-2</v>
+        <v>-0.2</v>
       </c>
       <c r="M44" s="2">
-        <v>-49.2</v>
+        <v>0.96</v>
       </c>
       <c r="N44" s="2">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="O44" s="3">
-        <v>1160</v>
+        <v>8972</v>
       </c>
     </row>
     <row r="45" spans="1:15">
@@ -3107,40 +3149,40 @@
         <v>17</v>
       </c>
       <c r="D45" s="2">
-        <v>0.42</v>
+        <v>0.02</v>
       </c>
       <c r="E45" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F45" s="2">
-        <v>1.32462</v>
+        <v>4997.44</v>
       </c>
       <c r="G45" s="2">
-        <v>1.3257</v>
+        <v>5021.56</v>
       </c>
       <c r="H45" s="2">
-        <v>1.32193</v>
+        <v>4907.23</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>152</v>
       </c>
       <c r="J45" s="2">
-        <v>1.32547</v>
+        <v>5004.36</v>
       </c>
       <c r="K45" s="2">
         <v>0</v>
       </c>
       <c r="L45" s="2">
-        <v>-2.1</v>
+        <v>-0.14</v>
       </c>
       <c r="M45" s="2">
-        <v>-35.7</v>
+        <v>-13.84</v>
       </c>
       <c r="N45" s="2">
-        <v>0</v>
+        <v>-6.9</v>
       </c>
       <c r="O45" s="3">
-        <v>5304</v>
+        <v>5470</v>
       </c>
     </row>
     <row r="46" spans="1:15">
@@ -3154,34 +3196,40 @@
         <v>17</v>
       </c>
       <c r="D46" s="2">
-        <v>0.42</v>
+        <v>0.65</v>
       </c>
       <c r="E46" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="F46" s="2">
-        <v>159.335</v>
+        <v>159.217</v>
+      </c>
+      <c r="G46" s="2">
+        <v>159.205</v>
+      </c>
+      <c r="H46" s="2">
+        <v>158.671</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>155</v>
       </c>
       <c r="J46" s="2">
-        <v>159.34</v>
+        <v>158.748</v>
       </c>
       <c r="K46" s="2">
         <v>0</v>
       </c>
       <c r="L46" s="2">
-        <v>-2.1</v>
+        <v>-3.26</v>
       </c>
       <c r="M46" s="2">
-        <v>-1.32</v>
+        <v>192.03</v>
       </c>
       <c r="N46" s="2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O46" s="3">
-        <v>5</v>
+        <v>21651</v>
       </c>
     </row>
     <row r="47" spans="1:15">
@@ -3192,43 +3240,43 @@
         <v>157</v>
       </c>
       <c r="C47" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D47" s="2">
-        <v>0.5</v>
+        <v>0.03</v>
       </c>
       <c r="E47" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F47" s="2">
-        <v>159.343</v>
+        <v>5013.0</v>
       </c>
       <c r="G47" s="2">
-        <v>159.188</v>
+        <v>5036.01</v>
       </c>
       <c r="H47" s="2">
-        <v>159.676</v>
+        <v>4938.12</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>158</v>
       </c>
       <c r="J47" s="2">
-        <v>159.231</v>
+        <v>5021.27</v>
       </c>
       <c r="K47" s="2">
         <v>0</v>
       </c>
       <c r="L47" s="2">
-        <v>-2.5</v>
+        <v>-0.22</v>
       </c>
       <c r="M47" s="2">
-        <v>-35.17</v>
+        <v>-24.81</v>
       </c>
       <c r="N47" s="2">
-        <v>-0.1</v>
+        <v>-8.3</v>
       </c>
       <c r="O47" s="3">
-        <v>3233</v>
+        <v>12894</v>
       </c>
     </row>
     <row r="48" spans="1:15">
@@ -3242,40 +3290,40 @@
         <v>17</v>
       </c>
       <c r="D48" s="2">
-        <v>0.29</v>
+        <v>0.03</v>
       </c>
       <c r="E48" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F48" s="2">
-        <v>1.33625</v>
+        <v>5009.64</v>
       </c>
       <c r="G48" s="2">
-        <v>1.33776</v>
+        <v>5039.17</v>
       </c>
       <c r="H48" s="2">
-        <v>1.33348</v>
+        <v>4945.32</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>161</v>
       </c>
       <c r="J48" s="2">
-        <v>1.33608</v>
+        <v>5023.34</v>
       </c>
       <c r="K48" s="2">
         <v>0</v>
       </c>
       <c r="L48" s="2">
-        <v>-1.46</v>
+        <v>-0.22</v>
       </c>
       <c r="M48" s="2">
-        <v>4.93</v>
+        <v>-41.1</v>
       </c>
       <c r="N48" s="2">
-        <v>0</v>
+        <v>-13.7</v>
       </c>
       <c r="O48" s="3">
-        <v>1925</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="49" spans="1:15">
@@ -3286,43 +3334,43 @@
         <v>163</v>
       </c>
       <c r="C49" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D49" s="2">
-        <v>0.45</v>
+        <v>0.02</v>
       </c>
       <c r="E49" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F49" s="2">
-        <v>159.158</v>
+        <v>5032.46</v>
       </c>
       <c r="G49" s="2">
-        <v>159.36</v>
+        <v>4996.97</v>
       </c>
       <c r="H49" s="2">
-        <v>158.563</v>
+        <v>5120.3</v>
       </c>
       <c r="I49" s="1" t="s">
         <v>164</v>
       </c>
       <c r="J49" s="2">
-        <v>159.365</v>
+        <v>5007.9</v>
       </c>
       <c r="K49" s="2">
         <v>0</v>
       </c>
       <c r="L49" s="2">
-        <v>-2.26</v>
+        <v>-0.14</v>
       </c>
       <c r="M49" s="2">
-        <v>-58.45</v>
+        <v>-49.12</v>
       </c>
       <c r="N49" s="2">
-        <v>-0.2</v>
+        <v>-24.6</v>
       </c>
       <c r="O49" s="3">
-        <v>5158</v>
+        <v>10248</v>
       </c>
     </row>
     <row r="50" spans="1:15">
@@ -3333,43 +3381,43 @@
         <v>166</v>
       </c>
       <c r="C50" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D50" s="2">
-        <v>0.02</v>
+        <v>0.4</v>
       </c>
       <c r="E50" t="s">
-        <v>22</v>
+        <v>107</v>
       </c>
       <c r="F50" s="2">
-        <v>5167.69</v>
+        <v>1.14738</v>
       </c>
       <c r="G50" s="2">
-        <v>5136.91</v>
+        <v>1.1486</v>
       </c>
       <c r="H50" s="2">
-        <v>5237.07</v>
+        <v>1.14474</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>167</v>
       </c>
       <c r="J50" s="2">
-        <v>5174.55</v>
+        <v>1.14861</v>
       </c>
       <c r="K50" s="2">
         <v>0</v>
       </c>
       <c r="L50" s="2">
-        <v>-0.14</v>
+        <v>-2</v>
       </c>
       <c r="M50" s="2">
-        <v>13.72</v>
+        <v>-49.2</v>
       </c>
       <c r="N50" s="2">
-        <v>6.9</v>
+        <v>0</v>
       </c>
       <c r="O50" s="3">
-        <v>15379</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="51" spans="1:15">
@@ -3383,40 +3431,40 @@
         <v>17</v>
       </c>
       <c r="D51" s="2">
-        <v>0.02</v>
+        <v>0.42</v>
       </c>
       <c r="E51" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F51" s="2">
-        <v>5167.72</v>
+        <v>1.32462</v>
       </c>
       <c r="G51" s="2">
-        <v>5183.68</v>
+        <v>1.3257</v>
       </c>
       <c r="H51" s="2">
-        <v>5088.57</v>
+        <v>1.32193</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>170</v>
       </c>
       <c r="J51" s="2">
-        <v>5155.96</v>
+        <v>1.32547</v>
       </c>
       <c r="K51" s="2">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2">
-        <v>-0.14</v>
+        <v>-2.1</v>
       </c>
       <c r="M51" s="2">
-        <v>23.52</v>
+        <v>-35.7</v>
       </c>
       <c r="N51" s="2">
-        <v>11.8</v>
+        <v>0</v>
       </c>
       <c r="O51" s="3">
-        <v>50331</v>
+        <v>5304</v>
       </c>
     </row>
     <row r="52" spans="1:15">
@@ -3430,40 +3478,34 @@
         <v>17</v>
       </c>
       <c r="D52" s="2">
-        <v>0.15</v>
+        <v>0.42</v>
       </c>
       <c r="E52" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F52" s="2">
-        <v>1.34062</v>
-      </c>
-      <c r="G52" s="2">
-        <v>1.34388</v>
-      </c>
-      <c r="H52" s="2">
-        <v>1.33251</v>
+        <v>159.335</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>173</v>
       </c>
       <c r="J52" s="2">
-        <v>1.34386</v>
+        <v>159.34</v>
       </c>
       <c r="K52" s="2">
         <v>0</v>
       </c>
       <c r="L52" s="2">
-        <v>-0.76</v>
+        <v>-2.1</v>
       </c>
       <c r="M52" s="2">
-        <v>-48.6</v>
+        <v>-1.32</v>
       </c>
       <c r="N52" s="2">
         <v>0</v>
       </c>
       <c r="O52" s="3">
-        <v>3555</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:15">
@@ -3474,43 +3516,43 @@
         <v>175</v>
       </c>
       <c r="C53" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D53" s="2">
-        <v>0.01</v>
+        <v>0.5</v>
       </c>
       <c r="E53" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F53" s="2">
-        <v>5165.53</v>
+        <v>159.343</v>
       </c>
       <c r="G53" s="2">
-        <v>5168.94</v>
+        <v>159.188</v>
       </c>
       <c r="H53" s="2">
-        <v>5287.9</v>
+        <v>159.676</v>
       </c>
       <c r="I53" s="1" t="s">
         <v>176</v>
       </c>
       <c r="J53" s="2">
-        <v>5185.4</v>
+        <v>159.231</v>
       </c>
       <c r="K53" s="2">
-        <v>-0.85</v>
+        <v>0</v>
       </c>
       <c r="L53" s="2">
-        <v>-0.08</v>
+        <v>-2.5</v>
       </c>
       <c r="M53" s="2">
-        <v>19.87</v>
+        <v>-35.17</v>
       </c>
       <c r="N53" s="2">
-        <v>19.9</v>
+        <v>-0.1</v>
       </c>
       <c r="O53" s="3">
-        <v>119287</v>
+        <v>3233</v>
       </c>
     </row>
     <row r="54" spans="1:15">
@@ -3521,43 +3563,43 @@
         <v>178</v>
       </c>
       <c r="C54" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D54" s="2">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="E54" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F54" s="2">
-        <v>1.3366</v>
+        <v>1.33625</v>
       </c>
       <c r="G54" s="2">
-        <v>1.33328</v>
+        <v>1.33776</v>
       </c>
       <c r="H54" s="2">
-        <v>1.34393</v>
+        <v>1.33348</v>
       </c>
       <c r="I54" s="1" t="s">
         <v>179</v>
       </c>
       <c r="J54" s="2">
-        <v>1.33599</v>
+        <v>1.33608</v>
       </c>
       <c r="K54" s="2">
         <v>0</v>
       </c>
       <c r="L54" s="2">
-        <v>-0.76</v>
+        <v>-1.46</v>
       </c>
       <c r="M54" s="2">
-        <v>-9.15</v>
+        <v>4.93</v>
       </c>
       <c r="N54" s="2">
         <v>0</v>
       </c>
       <c r="O54" s="3">
-        <v>25430</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="55" spans="1:15">
@@ -3571,40 +3613,40 @@
         <v>17</v>
       </c>
       <c r="D55" s="2">
-        <v>0.01</v>
+        <v>0.45</v>
       </c>
       <c r="E55" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F55" s="2">
-        <v>5133.69</v>
+        <v>159.158</v>
       </c>
       <c r="G55" s="2">
-        <v>5129.95</v>
+        <v>159.36</v>
       </c>
       <c r="H55" s="2">
-        <v>5017.48</v>
+        <v>158.563</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>182</v>
       </c>
       <c r="J55" s="2">
-        <v>5129.99</v>
+        <v>159.365</v>
       </c>
       <c r="K55" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2">
-        <v>-0.08</v>
+        <v>-2.26</v>
       </c>
       <c r="M55" s="2">
-        <v>3.7</v>
+        <v>-58.45</v>
       </c>
       <c r="N55" s="2">
-        <v>3.7</v>
+        <v>-0.2</v>
       </c>
       <c r="O55" s="3">
-        <v>43620</v>
+        <v>5158</v>
       </c>
     </row>
     <row r="56" spans="1:15">
@@ -3615,43 +3657,43 @@
         <v>184</v>
       </c>
       <c r="C56" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D56" s="2">
-        <v>0.22</v>
+        <v>0.02</v>
       </c>
       <c r="E56" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F56" s="2">
-        <v>156.295</v>
+        <v>5167.69</v>
       </c>
       <c r="G56" s="2">
-        <v>156.323</v>
+        <v>5136.91</v>
       </c>
       <c r="H56" s="2">
-        <v>157.627</v>
+        <v>5237.07</v>
       </c>
       <c r="I56" s="1" t="s">
         <v>185</v>
       </c>
       <c r="J56" s="2">
-        <v>157.017</v>
+        <v>5174.55</v>
       </c>
       <c r="K56" s="2">
         <v>0</v>
       </c>
       <c r="L56" s="2">
-        <v>-1.1</v>
+        <v>-0.14</v>
       </c>
       <c r="M56" s="2">
-        <v>101.16</v>
+        <v>13.72</v>
       </c>
       <c r="N56" s="2">
-        <v>0.7</v>
+        <v>6.9</v>
       </c>
       <c r="O56" s="3">
-        <v>15925</v>
+        <v>15379</v>
       </c>
     </row>
     <row r="57" spans="1:15">
@@ -3662,43 +3704,43 @@
         <v>187</v>
       </c>
       <c r="C57" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D57" s="2">
         <v>0.02</v>
       </c>
       <c r="E57" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F57" s="2">
-        <v>5191.98</v>
+        <v>5167.72</v>
       </c>
       <c r="G57" s="2">
-        <v>5161.5</v>
+        <v>5183.68</v>
       </c>
       <c r="H57" s="2">
-        <v>5279.36</v>
+        <v>5088.57</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>188</v>
       </c>
       <c r="J57" s="2">
-        <v>5174.77</v>
+        <v>5155.96</v>
       </c>
       <c r="K57" s="2">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="L57" s="2">
         <v>-0.14</v>
       </c>
       <c r="M57" s="2">
-        <v>-34.42</v>
+        <v>23.52</v>
       </c>
       <c r="N57" s="2">
-        <v>-17.2</v>
+        <v>11.8</v>
       </c>
       <c r="O57" s="3">
-        <v>29197</v>
+        <v>50331</v>
       </c>
     </row>
     <row r="58" spans="1:15">
@@ -3709,43 +3751,43 @@
         <v>190</v>
       </c>
       <c r="C58" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D58" s="2">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="E58" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F58" s="2">
-        <v>1.3534</v>
+        <v>1.34062</v>
       </c>
       <c r="G58" s="2">
-        <v>1.3539</v>
+        <v>1.34388</v>
       </c>
       <c r="H58" s="2">
-        <v>1.36038</v>
+        <v>1.33251</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>191</v>
       </c>
       <c r="J58" s="2">
-        <v>1.35389</v>
+        <v>1.34386</v>
       </c>
       <c r="K58" s="2">
-        <v>-2.77</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2">
-        <v>-0.8</v>
+        <v>-0.76</v>
       </c>
       <c r="M58" s="2">
-        <v>7.84</v>
+        <v>-48.6</v>
       </c>
       <c r="N58" s="2">
         <v>0</v>
       </c>
       <c r="O58" s="3">
-        <v>57837</v>
+        <v>3555</v>
       </c>
     </row>
     <row r="59" spans="1:15">
@@ -3756,43 +3798,43 @@
         <v>193</v>
       </c>
       <c r="C59" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D59" s="2">
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="E59" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="F59" s="2">
-        <v>155.883</v>
+        <v>5165.53</v>
       </c>
       <c r="G59" s="2">
-        <v>155.501</v>
+        <v>5168.94</v>
       </c>
       <c r="H59" s="2">
-        <v>157.591</v>
+        <v>5287.9</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>194</v>
       </c>
       <c r="J59" s="2">
-        <v>156.76</v>
+        <v>5185.4</v>
       </c>
       <c r="K59" s="2">
-        <v>0</v>
+        <v>-0.85</v>
       </c>
       <c r="L59" s="2">
-        <v>-1</v>
+        <v>-0.08</v>
       </c>
       <c r="M59" s="2">
-        <v>111.89</v>
+        <v>19.87</v>
       </c>
       <c r="N59" s="2">
-        <v>0.9</v>
+        <v>19.9</v>
       </c>
       <c r="O59" s="3">
-        <v>10543</v>
+        <v>119287</v>
       </c>
     </row>
     <row r="60" spans="1:15">
@@ -3803,28 +3845,28 @@
         <v>196</v>
       </c>
       <c r="C60" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D60" s="2">
         <v>0.15</v>
       </c>
       <c r="E60" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F60" s="2">
-        <v>1.34864</v>
+        <v>1.3366</v>
       </c>
       <c r="G60" s="2">
-        <v>1.35187</v>
+        <v>1.33328</v>
       </c>
       <c r="H60" s="2">
-        <v>1.33994</v>
+        <v>1.34393</v>
       </c>
       <c r="I60" s="1" t="s">
         <v>197</v>
       </c>
       <c r="J60" s="2">
-        <v>1.3492</v>
+        <v>1.33599</v>
       </c>
       <c r="K60" s="2">
         <v>0</v>
@@ -3833,13 +3875,13 @@
         <v>-0.76</v>
       </c>
       <c r="M60" s="2">
-        <v>-8.4</v>
+        <v>-9.15</v>
       </c>
       <c r="N60" s="2">
         <v>0</v>
       </c>
       <c r="O60" s="3">
-        <v>35458</v>
+        <v>25430</v>
       </c>
     </row>
     <row r="61" spans="1:15">
@@ -3853,119 +3895,119 @@
         <v>17</v>
       </c>
       <c r="D61" s="2">
-        <v>0.25</v>
+        <v>0.01</v>
       </c>
       <c r="E61" t="s">
+        <v>43</v>
+      </c>
+      <c r="F61" s="2">
+        <v>5133.69</v>
+      </c>
+      <c r="G61" s="2">
+        <v>5129.95</v>
+      </c>
+      <c r="H61" s="2">
+        <v>5017.48</v>
+      </c>
+      <c r="I61" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="F61" s="2">
-        <v>24742.45</v>
-      </c>
-      <c r="G61" s="2">
-        <v>24925.87</v>
-      </c>
-      <c r="H61" s="2">
-        <v>24377.7</v>
-      </c>
-      <c r="I61" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="J61" s="2">
-        <v>24844.75</v>
+        <v>5129.99</v>
       </c>
       <c r="K61" s="2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L61" s="2">
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="M61" s="2">
-        <v>-25.58</v>
+        <v>3.7</v>
       </c>
       <c r="N61" s="2">
-        <v>-102.3</v>
+        <v>3.7</v>
       </c>
       <c r="O61" s="3">
-        <v>11161</v>
+        <v>43620</v>
       </c>
     </row>
     <row r="62" spans="1:15">
       <c r="A62" t="s">
+        <v>201</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="C62" t="s">
+        <v>22</v>
+      </c>
+      <c r="D62" s="2">
+        <v>0.22</v>
+      </c>
+      <c r="E62" t="s">
+        <v>23</v>
+      </c>
+      <c r="F62" s="2">
+        <v>156.295</v>
+      </c>
+      <c r="G62" s="2">
+        <v>156.323</v>
+      </c>
+      <c r="H62" s="2">
+        <v>157.627</v>
+      </c>
+      <c r="I62" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C62" t="s">
-        <v>17</v>
-      </c>
-      <c r="D62" s="2">
-        <v>0.25</v>
-      </c>
-      <c r="E62" t="s">
-        <v>200</v>
-      </c>
-      <c r="F62" s="2">
-        <v>24731.38</v>
-      </c>
-      <c r="G62" s="2">
-        <v>24926.76</v>
-      </c>
-      <c r="H62" s="2">
-        <v>24316.56</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>204</v>
-      </c>
       <c r="J62" s="2">
-        <v>24826.88</v>
+        <v>157.017</v>
       </c>
       <c r="K62" s="2">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2">
-        <v>0</v>
+        <v>-1.1</v>
       </c>
       <c r="M62" s="2">
-        <v>-23.88</v>
+        <v>101.16</v>
       </c>
       <c r="N62" s="2">
-        <v>-95.5</v>
+        <v>0.7</v>
       </c>
       <c r="O62" s="3">
-        <v>35570</v>
+        <v>15925</v>
       </c>
     </row>
     <row r="63" spans="1:15">
       <c r="A63" t="s">
+        <v>204</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="B63" s="1" t="s">
-        <v>206</v>
-      </c>
       <c r="C63" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D63" s="2">
         <v>0.02</v>
       </c>
       <c r="E63" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F63" s="2">
-        <v>5013.18</v>
+        <v>5191.98</v>
       </c>
       <c r="G63" s="2">
-        <v>4981.37</v>
+        <v>5161.5</v>
       </c>
       <c r="H63" s="2">
-        <v>5119.17</v>
+        <v>5279.36</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J63" s="2">
-        <v>5020.44</v>
+        <v>5174.77</v>
       </c>
       <c r="K63" s="2">
         <v>0</v>
@@ -3974,200 +4016,482 @@
         <v>-0.14</v>
       </c>
       <c r="M63" s="2">
-        <v>14.52</v>
+        <v>-34.42</v>
       </c>
       <c r="N63" s="2">
-        <v>7.3</v>
+        <v>-17.2</v>
       </c>
       <c r="O63" s="3">
-        <v>17509</v>
+        <v>29197</v>
       </c>
     </row>
     <row r="64" spans="1:15">
       <c r="A64" t="s">
+        <v>207</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="C64" t="s">
+        <v>22</v>
+      </c>
+      <c r="D64" s="2">
+        <v>0.16</v>
+      </c>
+      <c r="E64" t="s">
+        <v>27</v>
+      </c>
+      <c r="F64" s="2">
+        <v>1.3534</v>
+      </c>
+      <c r="G64" s="2">
+        <v>1.3539</v>
+      </c>
+      <c r="H64" s="2">
+        <v>1.36038</v>
+      </c>
+      <c r="I64" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="C64" t="s">
-        <v>32</v>
-      </c>
-      <c r="D64" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="E64" t="s">
-        <v>70</v>
-      </c>
-      <c r="F64" s="2">
-        <v>153.574</v>
-      </c>
-      <c r="G64" s="2">
-        <v>153.59</v>
-      </c>
-      <c r="H64" s="2">
-        <v>154.652</v>
-      </c>
-      <c r="I64" s="1" t="s">
-        <v>210</v>
-      </c>
       <c r="J64" s="2">
-        <v>154.565</v>
+        <v>1.35389</v>
       </c>
       <c r="K64" s="2">
-        <v>0</v>
+        <v>-2.77</v>
       </c>
       <c r="L64" s="2">
-        <v>-0.76</v>
+        <v>-0.8</v>
       </c>
       <c r="M64" s="2">
-        <v>96.17</v>
+        <v>7.84</v>
       </c>
       <c r="N64" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O64" s="3">
-        <v>49948</v>
+        <v>57837</v>
       </c>
     </row>
     <row r="65" spans="1:15">
       <c r="A65" t="s">
+        <v>210</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="C65" t="s">
+        <v>22</v>
+      </c>
+      <c r="D65" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="E65" t="s">
+        <v>23</v>
+      </c>
+      <c r="F65" s="2">
+        <v>155.883</v>
+      </c>
+      <c r="G65" s="2">
+        <v>155.501</v>
+      </c>
+      <c r="H65" s="2">
+        <v>157.591</v>
+      </c>
+      <c r="I65" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="C65" t="s">
-        <v>32</v>
-      </c>
-      <c r="D65" s="2">
-        <v>0.21</v>
-      </c>
-      <c r="E65" t="s">
-        <v>70</v>
-      </c>
-      <c r="F65" s="2">
-        <v>153.618</v>
-      </c>
-      <c r="G65" s="2">
-        <v>153.263</v>
-      </c>
-      <c r="H65" s="2">
-        <v>154.408</v>
-      </c>
-      <c r="I65" s="1" t="s">
-        <v>213</v>
-      </c>
       <c r="J65" s="2">
-        <v>153.263</v>
+        <v>156.76</v>
       </c>
       <c r="K65" s="2">
         <v>0</v>
       </c>
       <c r="L65" s="2">
-        <v>-1.06</v>
+        <v>-1</v>
       </c>
       <c r="M65" s="2">
-        <v>-48.64</v>
+        <v>111.89</v>
       </c>
       <c r="N65" s="2">
-        <v>-0.4</v>
+        <v>0.9</v>
       </c>
       <c r="O65" s="3">
-        <v>12294</v>
+        <v>10543</v>
       </c>
     </row>
     <row r="66" spans="1:15">
       <c r="A66" t="s">
+        <v>213</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>215</v>
       </c>
       <c r="C66" t="s">
         <v>17</v>
       </c>
       <c r="D66" s="2">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="E66" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="F66" s="2">
-        <v>152.817</v>
+        <v>1.34864</v>
       </c>
       <c r="G66" s="2">
-        <v>153.213</v>
+        <v>1.35187</v>
       </c>
       <c r="H66" s="2">
-        <v>151.947</v>
+        <v>1.33994</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J66" s="2">
-        <v>153.213</v>
+        <v>1.3492</v>
       </c>
       <c r="K66" s="2">
         <v>0</v>
       </c>
       <c r="L66" s="2">
-        <v>-0.9</v>
+        <v>-0.76</v>
       </c>
       <c r="M66" s="2">
-        <v>-46.52</v>
+        <v>-8.4</v>
       </c>
       <c r="N66" s="2">
-        <v>-0.4</v>
+        <v>0</v>
       </c>
       <c r="O66" s="3">
-        <v>16480</v>
+        <v>35458</v>
       </c>
     </row>
     <row r="67" spans="1:15">
       <c r="A67" t="s">
+        <v>216</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>218</v>
       </c>
       <c r="C67" t="s">
         <v>17</v>
       </c>
       <c r="D67" s="2">
-        <v>0.21</v>
+        <v>0.25</v>
       </c>
       <c r="E67" t="s">
-        <v>89</v>
+        <v>218</v>
       </c>
       <c r="F67" s="2">
-        <v>1.18511</v>
+        <v>24742.45</v>
       </c>
       <c r="G67" s="2">
-        <v>1.18501</v>
+        <v>24925.87</v>
       </c>
       <c r="H67" s="2">
-        <v>1.18023</v>
+        <v>24377.7</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>219</v>
       </c>
       <c r="J67" s="2">
+        <v>24844.75</v>
+      </c>
+      <c r="K67" s="2">
+        <v>0</v>
+      </c>
+      <c r="L67" s="2">
+        <v>0</v>
+      </c>
+      <c r="M67" s="2">
+        <v>-25.58</v>
+      </c>
+      <c r="N67" s="2">
+        <v>-102.3</v>
+      </c>
+      <c r="O67" s="3">
+        <v>11161</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15">
+      <c r="A68" t="s">
+        <v>220</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C68" t="s">
+        <v>17</v>
+      </c>
+      <c r="D68" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E68" t="s">
+        <v>218</v>
+      </c>
+      <c r="F68" s="2">
+        <v>24731.38</v>
+      </c>
+      <c r="G68" s="2">
+        <v>24926.76</v>
+      </c>
+      <c r="H68" s="2">
+        <v>24316.56</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="J68" s="2">
+        <v>24826.88</v>
+      </c>
+      <c r="K68" s="2">
+        <v>0.06</v>
+      </c>
+      <c r="L68" s="2">
+        <v>0</v>
+      </c>
+      <c r="M68" s="2">
+        <v>-23.88</v>
+      </c>
+      <c r="N68" s="2">
+        <v>-95.5</v>
+      </c>
+      <c r="O68" s="3">
+        <v>35570</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15">
+      <c r="A69" t="s">
+        <v>223</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C69" t="s">
+        <v>22</v>
+      </c>
+      <c r="D69" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="E69" t="s">
+        <v>43</v>
+      </c>
+      <c r="F69" s="2">
+        <v>5013.18</v>
+      </c>
+      <c r="G69" s="2">
+        <v>4981.37</v>
+      </c>
+      <c r="H69" s="2">
+        <v>5119.17</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="J69" s="2">
+        <v>5020.44</v>
+      </c>
+      <c r="K69" s="2">
+        <v>0</v>
+      </c>
+      <c r="L69" s="2">
+        <v>-0.14</v>
+      </c>
+      <c r="M69" s="2">
+        <v>14.52</v>
+      </c>
+      <c r="N69" s="2">
+        <v>7.3</v>
+      </c>
+      <c r="O69" s="3">
+        <v>17509</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15">
+      <c r="A70" t="s">
+        <v>226</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C70" t="s">
+        <v>22</v>
+      </c>
+      <c r="D70" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="E70" t="s">
+        <v>23</v>
+      </c>
+      <c r="F70" s="2">
+        <v>153.574</v>
+      </c>
+      <c r="G70" s="2">
+        <v>153.59</v>
+      </c>
+      <c r="H70" s="2">
+        <v>154.652</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="J70" s="2">
+        <v>154.565</v>
+      </c>
+      <c r="K70" s="2">
+        <v>0</v>
+      </c>
+      <c r="L70" s="2">
+        <v>-0.76</v>
+      </c>
+      <c r="M70" s="2">
+        <v>96.17</v>
+      </c>
+      <c r="N70" s="2">
+        <v>1</v>
+      </c>
+      <c r="O70" s="3">
+        <v>49948</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15">
+      <c r="A71" t="s">
+        <v>229</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C71" t="s">
+        <v>22</v>
+      </c>
+      <c r="D71" s="2">
+        <v>0.21</v>
+      </c>
+      <c r="E71" t="s">
+        <v>23</v>
+      </c>
+      <c r="F71" s="2">
+        <v>153.618</v>
+      </c>
+      <c r="G71" s="2">
+        <v>153.263</v>
+      </c>
+      <c r="H71" s="2">
+        <v>154.408</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="J71" s="2">
+        <v>153.263</v>
+      </c>
+      <c r="K71" s="2">
+        <v>0</v>
+      </c>
+      <c r="L71" s="2">
+        <v>-1.06</v>
+      </c>
+      <c r="M71" s="2">
+        <v>-48.64</v>
+      </c>
+      <c r="N71" s="2">
+        <v>-0.4</v>
+      </c>
+      <c r="O71" s="3">
+        <v>12294</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15">
+      <c r="A72" t="s">
+        <v>232</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C72" t="s">
+        <v>17</v>
+      </c>
+      <c r="D72" s="2">
+        <v>0.18</v>
+      </c>
+      <c r="E72" t="s">
+        <v>23</v>
+      </c>
+      <c r="F72" s="2">
+        <v>152.817</v>
+      </c>
+      <c r="G72" s="2">
+        <v>153.213</v>
+      </c>
+      <c r="H72" s="2">
+        <v>151.947</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="J72" s="2">
+        <v>153.213</v>
+      </c>
+      <c r="K72" s="2">
+        <v>0</v>
+      </c>
+      <c r="L72" s="2">
+        <v>-0.9</v>
+      </c>
+      <c r="M72" s="2">
+        <v>-46.52</v>
+      </c>
+      <c r="N72" s="2">
+        <v>-0.4</v>
+      </c>
+      <c r="O72" s="3">
+        <v>16480</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15">
+      <c r="A73" t="s">
+        <v>235</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C73" t="s">
+        <v>17</v>
+      </c>
+      <c r="D73" s="2">
+        <v>0.21</v>
+      </c>
+      <c r="E73" t="s">
+        <v>107</v>
+      </c>
+      <c r="F73" s="2">
+        <v>1.18511</v>
+      </c>
+      <c r="G73" s="2">
+        <v>1.18501</v>
+      </c>
+      <c r="H73" s="2">
+        <v>1.18023</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="J73" s="2">
         <v>1.18447</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K73" s="2">
         <v>0.19</v>
       </c>
-      <c r="L67" s="2">
+      <c r="L73" s="2">
         <v>-1.06</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M73" s="2">
         <v>13.44</v>
       </c>
-      <c r="N67" s="2">
-        <v>0</v>
-      </c>
-      <c r="O67" s="3">
+      <c r="N73" s="2">
+        <v>0</v>
+      </c>
+      <c r="O73" s="3">
         <v>71443</v>
       </c>
     </row>

</xml_diff>